<commit_message>
Refresh test fixtures via canonical transaction-detail-workflow.ps1
Re-extracts all four Transaction Detail fixtures through
`Tools/queries/transaction-detail-workflow.ps1` so they consistently
carry the F4111 Ext column populated by the 2026-05 sproc update and
use the workflow's canonical output formatting (Text-formatted cells
that preserve "07    " as a string rather than Excel coercing it to
numeric 7).

- ic-1266229.xlsx (IC) — Pattern 5.4 + 5.14 secondary findings test
- ic-1293593.xlsx (IC) — Pattern 5.16 Mfg Cost Mismatch test
- im-1324740.xlsx (IM) — Pattern 5.4 Account Mismatch test
- pv-338338.xlsx (PV) — Pattern 5.17 Voucher Variance on Inventory
  test (F4111 empty per std-cost voucher behavior — Ext doesn't
  apply to this fixture)

No analyzer code changes; this just brings the fixtures in line with
the script's output shape, removing the ad-hoc Excel COM rebuild
I did earlier this session.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tools/_test_corpus/fixtures/ic-1266229.xlsx
+++ b/Tools/_test_corpus/fixtures/ic-1266229.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\source\repos\RapidReconciler-AI\.claude\worktrees\recursing-williamson-0f6630\Tools\_test_corpus\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCD0A5AF-5B13-4F8E-B28D-DE9909F4A903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{747A34D9-E54B-4321-B45B-0B323BC2A0F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="585" yWindow="735" windowWidth="16845" windowHeight="14640" xr2:uid="{45E83C48-B089-4028-A5DF-00FA188E7713}"/>
+    <workbookView xWindow="2220" yWindow="720" windowWidth="22275" windowHeight="14640" xr2:uid="{32070C4C-906D-4052-A6A9-BE3A0867A2BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Transaction Details" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="109">
-  <si>
-    <t>Transaction Details Generated Monday, May 18, 2026 04:45 PM</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="110">
+  <si>
+    <t>Transaction Details Generated Monday, May 18, 2026 11:01 PM</t>
   </si>
   <si>
     <t>Period</t>
@@ -176,13 +176,16 @@
     <t>0.000</t>
   </si>
   <si>
+    <t xml:space="preserve">07    </t>
+  </si>
+  <si>
     <t xml:space="preserve">Y     </t>
   </si>
   <si>
     <t xml:space="preserve">IDM         </t>
   </si>
   <si>
-    <t xml:space="preserve">468-35122-007            </t>
+    <t xml:space="preserve">468-35122-007                           </t>
   </si>
   <si>
     <t xml:space="preserve">WHS4                </t>
@@ -746,7 +749,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B51EEF5D-FB9D-4160-A585-517DB5965AD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF244B9-695C-4BC7-A8B5-AEC7D6F923E7}">
   <dimension ref="A1:AB48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1227,31 +1230,31 @@
         <v>44</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X6" s="1">
         <v>1985.68</v>
@@ -1266,12 +1269,12 @@
         <v>29</v>
       </c>
       <c r="AB6" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>40</v>
@@ -1283,16 +1286,16 @@
         <v>32</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>29</v>
@@ -1313,31 +1316,31 @@
         <v>44</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X7" s="1">
         <v>398.61</v>
@@ -1352,12 +1355,12 @@
         <v>29</v>
       </c>
       <c r="AB7" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>40</v>
@@ -1369,16 +1372,16 @@
         <v>32</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>29</v>
@@ -1399,31 +1402,31 @@
         <v>44</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X8" s="1">
         <v>433.24</v>
@@ -1438,12 +1441,12 @@
         <v>29</v>
       </c>
       <c r="AB8" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>40</v>
@@ -1455,16 +1458,16 @@
         <v>32</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>29</v>
@@ -1485,31 +1488,31 @@
         <v>44</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X9" s="1">
         <v>4579.95</v>
@@ -1524,12 +1527,12 @@
         <v>29</v>
       </c>
       <c r="AB9" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>40</v>
@@ -1541,16 +1544,16 @@
         <v>32</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>29</v>
@@ -1571,31 +1574,31 @@
         <v>44</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X10" s="1">
         <v>722.06</v>
@@ -1610,12 +1613,12 @@
         <v>29</v>
       </c>
       <c r="AB10" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>40</v>
@@ -1627,16 +1630,16 @@
         <v>32</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>29</v>
@@ -1657,31 +1660,31 @@
         <v>44</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X11" s="1">
         <v>144.41</v>
@@ -1696,12 +1699,12 @@
         <v>29</v>
       </c>
       <c r="AB11" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>40</v>
@@ -1713,16 +1716,16 @@
         <v>32</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>29</v>
@@ -1743,31 +1746,31 @@
         <v>44</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X12" s="1">
         <v>1458.86</v>
@@ -1782,7 +1785,7 @@
         <v>29</v>
       </c>
       <c r="AB12" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
@@ -1793,7 +1796,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>29</v>
@@ -1865,7 +1868,7 @@
         <v>29</v>
       </c>
       <c r="AA13" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AB13" s="1" t="s">
         <v>29</v>
@@ -1876,7 +1879,7 @@
         <v>29</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>29</v>
@@ -1962,10 +1965,10 @@
         <v>39</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>32</v>
@@ -1983,10 +1986,10 @@
         <v>43</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>34</v>
@@ -1998,13 +2001,13 @@
         <v>35</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q15" s="1" t="s">
         <v>29</v>
@@ -2040,39 +2043,39 @@
         <v>29</v>
       </c>
       <c r="AB15" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>34</v>
@@ -2084,13 +2087,13 @@
         <v>35</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q16" s="1" t="s">
         <v>29</v>
@@ -2126,39 +2129,39 @@
         <v>29</v>
       </c>
       <c r="AB16" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>34</v>
@@ -2170,13 +2173,13 @@
         <v>35</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q17" s="1" t="s">
         <v>29</v>
@@ -2212,39 +2215,39 @@
         <v>29</v>
       </c>
       <c r="AB17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>34</v>
@@ -2256,13 +2259,13 @@
         <v>35</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q18" s="1" t="s">
         <v>29</v>
@@ -2298,39 +2301,39 @@
         <v>29</v>
       </c>
       <c r="AB18" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>34</v>
@@ -2342,13 +2345,13 @@
         <v>35</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="1" t="s">
         <v>29</v>
@@ -2384,39 +2387,39 @@
         <v>29</v>
       </c>
       <c r="AB19" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>34</v>
@@ -2428,13 +2431,13 @@
         <v>35</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q20" s="1" t="s">
         <v>29</v>
@@ -2470,39 +2473,39 @@
         <v>29</v>
       </c>
       <c r="AB20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>34</v>
@@ -2514,13 +2517,13 @@
         <v>35</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q21" s="1" t="s">
         <v>29</v>
@@ -2556,7 +2559,7 @@
         <v>29</v>
       </c>
       <c r="AB21" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
@@ -2567,7 +2570,7 @@
         <v>29</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>29</v>
@@ -2639,10 +2642,10 @@
         <v>29</v>
       </c>
       <c r="AA22" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AB22" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.25">
@@ -2736,7 +2739,7 @@
         <v>29</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>29</v>
@@ -2908,7 +2911,7 @@
         <v>29</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>29</v>
@@ -2997,7 +3000,7 @@
         <v>40</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>32</v>
@@ -3015,7 +3018,7 @@
         <v>43</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>33</v>
@@ -3080,10 +3083,10 @@
         <v>39</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>32</v>
@@ -3101,7 +3104,7 @@
         <v>43</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>33</v>
@@ -3163,13 +3166,13 @@
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>32</v>
@@ -3184,10 +3187,10 @@
         <v>29</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>33</v>
@@ -3249,13 +3252,13 @@
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>32</v>
@@ -3270,10 +3273,10 @@
         <v>29</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>33</v>
@@ -3335,13 +3338,13 @@
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>32</v>
@@ -3356,10 +3359,10 @@
         <v>29</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>33</v>
@@ -3421,13 +3424,13 @@
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>32</v>
@@ -3442,10 +3445,10 @@
         <v>29</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>33</v>
@@ -3507,13 +3510,13 @@
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>32</v>
@@ -3528,10 +3531,10 @@
         <v>29</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>33</v>
@@ -3593,13 +3596,13 @@
     </row>
     <row r="34" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>32</v>
@@ -3614,10 +3617,10 @@
         <v>29</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>33</v>
@@ -3679,13 +3682,13 @@
     </row>
     <row r="35" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>32</v>
@@ -3700,10 +3703,10 @@
         <v>29</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>33</v>
@@ -3765,13 +3768,13 @@
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>32</v>
@@ -3786,10 +3789,10 @@
         <v>29</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>33</v>
@@ -3851,13 +3854,13 @@
     </row>
     <row r="37" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>32</v>
@@ -3872,10 +3875,10 @@
         <v>29</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>33</v>
@@ -3937,13 +3940,13 @@
     </row>
     <row r="38" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>32</v>
@@ -3958,10 +3961,10 @@
         <v>29</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>33</v>
@@ -4023,13 +4026,13 @@
     </row>
     <row r="39" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>32</v>
@@ -4044,10 +4047,10 @@
         <v>29</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>33</v>
@@ -4109,13 +4112,13 @@
     </row>
     <row r="40" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>32</v>
@@ -4130,10 +4133,10 @@
         <v>29</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J40" s="1" t="s">
         <v>33</v>
@@ -4201,7 +4204,7 @@
         <v>29</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>29</v>
@@ -4273,7 +4276,7 @@
         <v>-0.04</v>
       </c>
       <c r="AA41" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AB41" s="1" t="s">
         <v>37</v>
@@ -4370,7 +4373,7 @@
         <v>29</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>29</v>
@@ -4456,10 +4459,10 @@
         <v>29</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>4</v>
@@ -4480,10 +4483,10 @@
         <v>29</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>29</v>
@@ -4545,7 +4548,7 @@
         <v>40</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>32</v>
@@ -4566,16 +4569,16 @@
         <v>29</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L45" s="1" t="s">
         <v>29</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>29</v>
@@ -4714,10 +4717,10 @@
         <v>29</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>4</v>
@@ -4738,10 +4741,10 @@
         <v>29</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L47" s="1" t="s">
         <v>29</v>
@@ -4803,7 +4806,7 @@
         <v>40</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>32</v>
@@ -4824,7 +4827,7 @@
         <v>29</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K48" s="1" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Refresh test fixtures via canonical transaction-detail-workflow.ps1 (#65)
Re-extracts all four Transaction Detail fixtures through
`Tools/queries/transaction-detail-workflow.ps1` so they consistently
carry the F4111 Ext column populated by the 2026-05 sproc update and
use the workflow's canonical output formatting (Text-formatted cells
that preserve "07    " as a string rather than Excel coercing it to
numeric 7).

- ic-1266229.xlsx (IC) — Pattern 5.4 + 5.14 secondary findings test
- ic-1293593.xlsx (IC) — Pattern 5.16 Mfg Cost Mismatch test
- im-1324740.xlsx (IM) — Pattern 5.4 Account Mismatch test
- pv-338338.xlsx (PV) — Pattern 5.17 Voucher Variance on Inventory
  test (F4111 empty per std-cost voucher behavior — Ext doesn't
  apply to this fixture)

No analyzer code changes; this just brings the fixtures in line with
the script's output shape, removing the ad-hoc Excel COM rebuild
I did earlier this session.

Co-authored-by: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tools/_test_corpus/fixtures/ic-1266229.xlsx
+++ b/Tools/_test_corpus/fixtures/ic-1266229.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\source\repos\RapidReconciler-AI\.claude\worktrees\recursing-williamson-0f6630\Tools\_test_corpus\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCD0A5AF-5B13-4F8E-B28D-DE9909F4A903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{747A34D9-E54B-4321-B45B-0B323BC2A0F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="585" yWindow="735" windowWidth="16845" windowHeight="14640" xr2:uid="{45E83C48-B089-4028-A5DF-00FA188E7713}"/>
+    <workbookView xWindow="2220" yWindow="720" windowWidth="22275" windowHeight="14640" xr2:uid="{32070C4C-906D-4052-A6A9-BE3A0867A2BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Transaction Details" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="109">
-  <si>
-    <t>Transaction Details Generated Monday, May 18, 2026 04:45 PM</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="110">
+  <si>
+    <t>Transaction Details Generated Monday, May 18, 2026 11:01 PM</t>
   </si>
   <si>
     <t>Period</t>
@@ -176,13 +176,16 @@
     <t>0.000</t>
   </si>
   <si>
+    <t xml:space="preserve">07    </t>
+  </si>
+  <si>
     <t xml:space="preserve">Y     </t>
   </si>
   <si>
     <t xml:space="preserve">IDM         </t>
   </si>
   <si>
-    <t xml:space="preserve">468-35122-007            </t>
+    <t xml:space="preserve">468-35122-007                           </t>
   </si>
   <si>
     <t xml:space="preserve">WHS4                </t>
@@ -746,7 +749,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B51EEF5D-FB9D-4160-A585-517DB5965AD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF244B9-695C-4BC7-A8B5-AEC7D6F923E7}">
   <dimension ref="A1:AB48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1227,31 +1230,31 @@
         <v>44</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X6" s="1">
         <v>1985.68</v>
@@ -1266,12 +1269,12 @@
         <v>29</v>
       </c>
       <c r="AB6" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>40</v>
@@ -1283,16 +1286,16 @@
         <v>32</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>29</v>
@@ -1313,31 +1316,31 @@
         <v>44</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X7" s="1">
         <v>398.61</v>
@@ -1352,12 +1355,12 @@
         <v>29</v>
       </c>
       <c r="AB7" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>40</v>
@@ -1369,16 +1372,16 @@
         <v>32</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>29</v>
@@ -1399,31 +1402,31 @@
         <v>44</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X8" s="1">
         <v>433.24</v>
@@ -1438,12 +1441,12 @@
         <v>29</v>
       </c>
       <c r="AB8" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>40</v>
@@ -1455,16 +1458,16 @@
         <v>32</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>29</v>
@@ -1485,31 +1488,31 @@
         <v>44</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X9" s="1">
         <v>4579.95</v>
@@ -1524,12 +1527,12 @@
         <v>29</v>
       </c>
       <c r="AB9" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>40</v>
@@ -1541,16 +1544,16 @@
         <v>32</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>29</v>
@@ -1571,31 +1574,31 @@
         <v>44</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X10" s="1">
         <v>722.06</v>
@@ -1610,12 +1613,12 @@
         <v>29</v>
       </c>
       <c r="AB10" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>40</v>
@@ -1627,16 +1630,16 @@
         <v>32</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>29</v>
@@ -1657,31 +1660,31 @@
         <v>44</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X11" s="1">
         <v>144.41</v>
@@ -1696,12 +1699,12 @@
         <v>29</v>
       </c>
       <c r="AB11" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>40</v>
@@ -1713,16 +1716,16 @@
         <v>32</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>42</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>29</v>
@@ -1743,31 +1746,31 @@
         <v>44</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X12" s="1">
         <v>1458.86</v>
@@ -1782,7 +1785,7 @@
         <v>29</v>
       </c>
       <c r="AB12" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
@@ -1793,7 +1796,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>29</v>
@@ -1865,7 +1868,7 @@
         <v>29</v>
       </c>
       <c r="AA13" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AB13" s="1" t="s">
         <v>29</v>
@@ -1876,7 +1879,7 @@
         <v>29</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>29</v>
@@ -1962,10 +1965,10 @@
         <v>39</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>32</v>
@@ -1983,10 +1986,10 @@
         <v>43</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>34</v>
@@ -1998,13 +2001,13 @@
         <v>35</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q15" s="1" t="s">
         <v>29</v>
@@ -2040,39 +2043,39 @@
         <v>29</v>
       </c>
       <c r="AB15" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>34</v>
@@ -2084,13 +2087,13 @@
         <v>35</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q16" s="1" t="s">
         <v>29</v>
@@ -2126,39 +2129,39 @@
         <v>29</v>
       </c>
       <c r="AB16" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>34</v>
@@ -2170,13 +2173,13 @@
         <v>35</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q17" s="1" t="s">
         <v>29</v>
@@ -2212,39 +2215,39 @@
         <v>29</v>
       </c>
       <c r="AB17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>34</v>
@@ -2256,13 +2259,13 @@
         <v>35</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q18" s="1" t="s">
         <v>29</v>
@@ -2298,39 +2301,39 @@
         <v>29</v>
       </c>
       <c r="AB18" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>34</v>
@@ -2342,13 +2345,13 @@
         <v>35</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="1" t="s">
         <v>29</v>
@@ -2384,39 +2387,39 @@
         <v>29</v>
       </c>
       <c r="AB19" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>34</v>
@@ -2428,13 +2431,13 @@
         <v>35</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q20" s="1" t="s">
         <v>29</v>
@@ -2470,39 +2473,39 @@
         <v>29</v>
       </c>
       <c r="AB20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>34</v>
@@ -2514,13 +2517,13 @@
         <v>35</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q21" s="1" t="s">
         <v>29</v>
@@ -2556,7 +2559,7 @@
         <v>29</v>
       </c>
       <c r="AB21" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
@@ -2567,7 +2570,7 @@
         <v>29</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>29</v>
@@ -2639,10 +2642,10 @@
         <v>29</v>
       </c>
       <c r="AA22" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AB22" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.25">
@@ -2736,7 +2739,7 @@
         <v>29</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>29</v>
@@ -2908,7 +2911,7 @@
         <v>29</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>29</v>
@@ -2997,7 +3000,7 @@
         <v>40</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>32</v>
@@ -3015,7 +3018,7 @@
         <v>43</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>33</v>
@@ -3080,10 +3083,10 @@
         <v>39</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>32</v>
@@ -3101,7 +3104,7 @@
         <v>43</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>33</v>
@@ -3163,13 +3166,13 @@
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>32</v>
@@ -3184,10 +3187,10 @@
         <v>29</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>33</v>
@@ -3249,13 +3252,13 @@
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>32</v>
@@ -3270,10 +3273,10 @@
         <v>29</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>33</v>
@@ -3335,13 +3338,13 @@
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>32</v>
@@ -3356,10 +3359,10 @@
         <v>29</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>33</v>
@@ -3421,13 +3424,13 @@
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>32</v>
@@ -3442,10 +3445,10 @@
         <v>29</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>33</v>
@@ -3507,13 +3510,13 @@
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>32</v>
@@ -3528,10 +3531,10 @@
         <v>29</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>33</v>
@@ -3593,13 +3596,13 @@
     </row>
     <row r="34" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>32</v>
@@ -3614,10 +3617,10 @@
         <v>29</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>33</v>
@@ -3679,13 +3682,13 @@
     </row>
     <row r="35" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>32</v>
@@ -3700,10 +3703,10 @@
         <v>29</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>33</v>
@@ -3765,13 +3768,13 @@
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>32</v>
@@ -3786,10 +3789,10 @@
         <v>29</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>33</v>
@@ -3851,13 +3854,13 @@
     </row>
     <row r="37" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>32</v>
@@ -3872,10 +3875,10 @@
         <v>29</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>33</v>
@@ -3937,13 +3940,13 @@
     </row>
     <row r="38" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>32</v>
@@ -3958,10 +3961,10 @@
         <v>29</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>33</v>
@@ -4023,13 +4026,13 @@
     </row>
     <row r="39" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>32</v>
@@ -4044,10 +4047,10 @@
         <v>29</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>33</v>
@@ -4109,13 +4112,13 @@
     </row>
     <row r="40" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>32</v>
@@ -4130,10 +4133,10 @@
         <v>29</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J40" s="1" t="s">
         <v>33</v>
@@ -4201,7 +4204,7 @@
         <v>29</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>29</v>
@@ -4273,7 +4276,7 @@
         <v>-0.04</v>
       </c>
       <c r="AA41" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AB41" s="1" t="s">
         <v>37</v>
@@ -4370,7 +4373,7 @@
         <v>29</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>29</v>
@@ -4456,10 +4459,10 @@
         <v>29</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>4</v>
@@ -4480,10 +4483,10 @@
         <v>29</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>29</v>
@@ -4545,7 +4548,7 @@
         <v>40</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>32</v>
@@ -4566,16 +4569,16 @@
         <v>29</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L45" s="1" t="s">
         <v>29</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>29</v>
@@ -4714,10 +4717,10 @@
         <v>29</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>4</v>
@@ -4738,10 +4741,10 @@
         <v>29</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L47" s="1" t="s">
         <v>29</v>
@@ -4803,7 +4806,7 @@
         <v>40</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>32</v>
@@ -4824,7 +4827,7 @@
         <v>29</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K48" s="1" t="s">
         <v>34</v>

</xml_diff>